<commit_message>
Show current ranking and other refactorings
</commit_message>
<xml_diff>
--- a/Templates/StartListTT.xlsx
+++ b/Templates/StartListTT.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8355" windowHeight="9510"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8352" windowHeight="9516"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgabenliste" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="168" formatCode="&quot;Erledigt&quot;;&quot;&quot;;&quot;&quot;"/>
-    <numFmt numFmtId="169" formatCode="mm:ss.0;@"/>
+    <numFmt numFmtId="169" formatCode="h:mm:ss;@"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -228,7 +228,7 @@
       <alignment horizontal="right" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -242,9 +242,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -265,6 +262,12 @@
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Datum" xfId="8"/>
@@ -280,84 +283,7 @@
     <cellStyle name="Währung" xfId="5" builtinId="4" customBuiltin="1"/>
     <cellStyle name="Währung [0]" xfId="6" builtinId="7" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="31">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="26">
     <dxf>
       <font>
         <b val="0"/>
@@ -372,7 +298,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="169" formatCode="mm:ss.0;@"/>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -388,6 +314,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -403,6 +330,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -418,6 +346,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="169" formatCode="h:mm:ss;@"/>
     </dxf>
     <dxf>
       <font>
@@ -469,6 +398,48 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -615,20 +586,20 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="Aufgabenliste" defaultPivotStyle="PivotStyleLight2">
     <tableStyle name="Aufgabenlisten-Pivot" table="0" count="11">
-      <tableStyleElement type="headerRow" dxfId="30"/>
-      <tableStyleElement type="totalRow" dxfId="29"/>
-      <tableStyleElement type="firstRowStripe" dxfId="28"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="27"/>
-      <tableStyleElement type="firstSubtotalColumn" dxfId="26"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="25"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="24"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="23"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="22"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="21"/>
-      <tableStyleElement type="pageFieldValues" dxfId="20"/>
+      <tableStyleElement type="headerRow" dxfId="25"/>
+      <tableStyleElement type="totalRow" dxfId="24"/>
+      <tableStyleElement type="firstRowStripe" dxfId="23"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="22"/>
+      <tableStyleElement type="firstSubtotalColumn" dxfId="21"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="20"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="19"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="18"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="17"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="16"/>
+      <tableStyleElement type="pageFieldValues" dxfId="15"/>
     </tableStyle>
     <tableStyle name="Aufgabenliste" pivot="0" count="1">
-      <tableStyleElement type="wholeTable" dxfId="19"/>
+      <tableStyleElement type="wholeTable" dxfId="14"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -643,13 +614,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ergebnisliste" displayName="Ergebnisliste" ref="A1:E2" insertRow="1" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ergebnisliste" displayName="Ergebnisliste" ref="A1:E2" insertRow="1" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6">
   <tableColumns count="5">
-    <tableColumn id="5" name="Start#" dataDxfId="15"/>
-    <tableColumn id="1" name="Name, Vorname" dataDxfId="14" dataCellStyle="Standard"/>
-    <tableColumn id="3" name="Verein" dataDxfId="13" dataCellStyle="Standard"/>
-    <tableColumn id="4" name="Team" dataDxfId="12" dataCellStyle="Standard"/>
-    <tableColumn id="6" name="Startzeit" dataDxfId="11" dataCellStyle="Datum"/>
+    <tableColumn id="5" name="Start#" dataDxfId="4"/>
+    <tableColumn id="1" name="Name, Vorname" dataDxfId="2" dataCellStyle="Standard"/>
+    <tableColumn id="3" name="Verein" dataDxfId="1" dataCellStyle="Standard"/>
+    <tableColumn id="4" name="Team" dataDxfId="0" dataCellStyle="Standard"/>
+    <tableColumn id="6" name="Startzeit" dataDxfId="3" dataCellStyle="Datum"/>
   </tableColumns>
   <tableStyleInfo name="Aufgabenliste" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
   <extLst>
@@ -892,1217 +863,1217 @@
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.54296875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.81640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" style="11" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="13.90625" style="10" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="9"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
+      <c r="A3" s="6"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="9"/>
+      <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
+      <c r="A4" s="6"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
-      <c r="E4" s="9"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
+      <c r="A6" s="6"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="9"/>
+      <c r="E6" s="8"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="9"/>
+      <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-      <c r="E8" s="9"/>
+      <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="9"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-      <c r="E10" s="9"/>
+      <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-      <c r="E11" s="9"/>
+      <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="9"/>
+      <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="9"/>
+      <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="9"/>
+      <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
-      <c r="E15" s="9"/>
+      <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
-      <c r="E16" s="9"/>
+      <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
-      <c r="E17" s="9"/>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
-      <c r="E18" s="9"/>
+      <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
-      <c r="E19" s="9"/>
+      <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
-      <c r="E22" s="9"/>
+      <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
-      <c r="E23" s="9"/>
+      <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="E24" s="10"/>
+      <c r="E24" s="9"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="9"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
-      <c r="E26" s="10"/>
+      <c r="E26" s="9"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
-      <c r="E27" s="10"/>
+      <c r="E27" s="9"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="9"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
-      <c r="E29" s="10"/>
+      <c r="E29" s="9"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
-      <c r="E30" s="10"/>
+      <c r="E30" s="9"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
-      <c r="E31" s="10"/>
+      <c r="E31" s="9"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
-      <c r="E32" s="10"/>
+      <c r="E32" s="9"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
-      <c r="E33" s="10"/>
+      <c r="E33" s="9"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
-      <c r="E34" s="10"/>
+      <c r="E34" s="9"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
-      <c r="E35" s="10"/>
+      <c r="E35" s="9"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
-      <c r="E36" s="10"/>
+      <c r="E36" s="9"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="10"/>
+      <c r="E37" s="9"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
-      <c r="E38" s="10"/>
+      <c r="E38" s="9"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
-      <c r="E39" s="10"/>
+      <c r="E39" s="9"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
-      <c r="E40" s="10"/>
+      <c r="E40" s="9"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
-      <c r="E41" s="10"/>
+      <c r="E41" s="9"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
-      <c r="E42" s="10"/>
+      <c r="E42" s="9"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
-      <c r="E43" s="10"/>
+      <c r="E43" s="9"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
-      <c r="E44" s="10"/>
+      <c r="E44" s="9"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
-      <c r="E45" s="10"/>
+      <c r="E45" s="9"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
-      <c r="E46" s="10"/>
+      <c r="E46" s="9"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
-      <c r="E47" s="10"/>
+      <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
-      <c r="E48" s="10"/>
+      <c r="E48" s="9"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
-      <c r="E49" s="10"/>
+      <c r="E49" s="9"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
-      <c r="E50" s="10"/>
+      <c r="E50" s="9"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
-      <c r="E51" s="10"/>
+      <c r="E51" s="9"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
-      <c r="E52" s="10"/>
+      <c r="E52" s="9"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
-      <c r="E53" s="10"/>
+      <c r="E53" s="9"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
-      <c r="E54" s="10"/>
+      <c r="E54" s="9"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
-      <c r="E55" s="10"/>
+      <c r="E55" s="9"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
-      <c r="E56" s="10"/>
+      <c r="E56" s="9"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
-      <c r="E57" s="10"/>
+      <c r="E57" s="9"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
-      <c r="E58" s="10"/>
+      <c r="E58" s="9"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
-      <c r="E59" s="10"/>
+      <c r="E59" s="9"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
-      <c r="E60" s="10"/>
+      <c r="E60" s="9"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
-      <c r="E61" s="10"/>
+      <c r="E61" s="9"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
-      <c r="E62" s="10"/>
+      <c r="E62" s="9"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
-      <c r="E63" s="10"/>
+      <c r="E63" s="9"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
-      <c r="E64" s="10"/>
+      <c r="E64" s="9"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
-      <c r="E65" s="10"/>
+      <c r="E65" s="9"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
-      <c r="E66" s="10"/>
+      <c r="E66" s="9"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
-      <c r="E67" s="10"/>
+      <c r="E67" s="9"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
-      <c r="E68" s="10"/>
+      <c r="E68" s="9"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
-      <c r="E69" s="10"/>
+      <c r="E69" s="9"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
-      <c r="E70" s="10"/>
+      <c r="E70" s="9"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
-      <c r="E71" s="10"/>
+      <c r="E71" s="9"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
-      <c r="E72" s="10"/>
+      <c r="E72" s="9"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
-      <c r="E73" s="10"/>
+      <c r="E73" s="9"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
-      <c r="E74" s="10"/>
+      <c r="E74" s="9"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
-      <c r="E75" s="10"/>
+      <c r="E75" s="9"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
-      <c r="E76" s="10"/>
+      <c r="E76" s="9"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
-      <c r="E77" s="10"/>
+      <c r="E77" s="9"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
-      <c r="E78" s="10"/>
+      <c r="E78" s="9"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
-      <c r="E79" s="10"/>
+      <c r="E79" s="9"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
-      <c r="E80" s="10"/>
+      <c r="E80" s="9"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
-      <c r="E81" s="10"/>
+      <c r="E81" s="9"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
-      <c r="E82" s="10"/>
+      <c r="E82" s="9"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
-      <c r="E83" s="10"/>
+      <c r="E83" s="9"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
-      <c r="E84" s="10"/>
+      <c r="E84" s="9"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
-      <c r="E85" s="10"/>
+      <c r="E85" s="9"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
-      <c r="E86" s="10"/>
+      <c r="E86" s="9"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
-      <c r="E87" s="10"/>
+      <c r="E87" s="9"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
-      <c r="E88" s="10"/>
+      <c r="E88" s="9"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
-      <c r="E89" s="10"/>
+      <c r="E89" s="9"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
-      <c r="E90" s="10"/>
+      <c r="E90" s="9"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
-      <c r="E91" s="10"/>
+      <c r="E91" s="9"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
-      <c r="E92" s="10"/>
+      <c r="E92" s="9"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
-      <c r="E93" s="10"/>
+      <c r="E93" s="9"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
-      <c r="E94" s="10"/>
+      <c r="E94" s="9"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
-      <c r="E95" s="10"/>
+      <c r="E95" s="9"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
-      <c r="E96" s="10"/>
+      <c r="E96" s="9"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
-      <c r="E97" s="10"/>
+      <c r="E97" s="9"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
-      <c r="E98" s="10"/>
+      <c r="E98" s="9"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
-      <c r="E99" s="10"/>
+      <c r="E99" s="9"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
-      <c r="E100" s="10"/>
+      <c r="E100" s="9"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
-      <c r="E101" s="10"/>
+      <c r="E101" s="9"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
-      <c r="E102" s="10"/>
+      <c r="E102" s="9"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
-      <c r="E103" s="10"/>
+      <c r="E103" s="9"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
-      <c r="E104" s="10"/>
+      <c r="E104" s="9"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
-      <c r="E105" s="10"/>
+      <c r="E105" s="9"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
-      <c r="E106" s="10"/>
+      <c r="E106" s="9"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
-      <c r="E107" s="10"/>
+      <c r="E107" s="9"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
-      <c r="E108" s="10"/>
+      <c r="E108" s="9"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
-      <c r="E109" s="10"/>
+      <c r="E109" s="9"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
-      <c r="E110" s="10"/>
+      <c r="E110" s="9"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
-      <c r="E111" s="10"/>
+      <c r="E111" s="9"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
-      <c r="E112" s="10"/>
+      <c r="E112" s="9"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
-      <c r="E113" s="10"/>
+      <c r="E113" s="9"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
-      <c r="E114" s="10"/>
+      <c r="E114" s="9"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
-      <c r="E115" s="10"/>
+      <c r="E115" s="9"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
-      <c r="E116" s="10"/>
+      <c r="E116" s="9"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
-      <c r="E117" s="10"/>
+      <c r="E117" s="9"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
-      <c r="E118" s="10"/>
+      <c r="E118" s="9"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
-      <c r="E119" s="10"/>
+      <c r="E119" s="9"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
-      <c r="E120" s="10"/>
+      <c r="E120" s="9"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
-      <c r="E121" s="10"/>
+      <c r="E121" s="9"/>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="3"/>
       <c r="D122" s="3"/>
-      <c r="E122" s="10"/>
+      <c r="E122" s="9"/>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
-      <c r="E123" s="10"/>
+      <c r="E123" s="9"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
-      <c r="E124" s="10"/>
+      <c r="E124" s="9"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
-      <c r="E125" s="10"/>
+      <c r="E125" s="9"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
-      <c r="E126" s="10"/>
+      <c r="E126" s="9"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
-      <c r="E127" s="10"/>
+      <c r="E127" s="9"/>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
-      <c r="E128" s="10"/>
+      <c r="E128" s="9"/>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
-      <c r="E129" s="10"/>
+      <c r="E129" s="9"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
-      <c r="E130" s="10"/>
+      <c r="E130" s="9"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
-      <c r="E131" s="10"/>
+      <c r="E131" s="9"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
-      <c r="E132" s="10"/>
+      <c r="E132" s="9"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
-      <c r="E133" s="10"/>
+      <c r="E133" s="9"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
-      <c r="E134" s="10"/>
+      <c r="E134" s="9"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
-      <c r="E135" s="10"/>
+      <c r="E135" s="9"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
-      <c r="E136" s="10"/>
+      <c r="E136" s="9"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="3"/>
       <c r="D137" s="3"/>
-      <c r="E137" s="10"/>
+      <c r="E137" s="9"/>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="3"/>
       <c r="D138" s="3"/>
-      <c r="E138" s="10"/>
+      <c r="E138" s="9"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
-      <c r="E139" s="10"/>
+      <c r="E139" s="9"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
-      <c r="E140" s="10"/>
+      <c r="E140" s="9"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="3"/>
       <c r="D141" s="3"/>
-      <c r="E141" s="10"/>
+      <c r="E141" s="9"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="3"/>
       <c r="D142" s="3"/>
-      <c r="E142" s="10"/>
+      <c r="E142" s="9"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
-      <c r="E143" s="10"/>
+      <c r="E143" s="9"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
-      <c r="E144" s="10"/>
+      <c r="E144" s="9"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
-      <c r="E145" s="10"/>
+      <c r="E145" s="9"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="3"/>
       <c r="D146" s="3"/>
-      <c r="E146" s="10"/>
+      <c r="E146" s="9"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
-      <c r="E147" s="10"/>
+      <c r="E147" s="9"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
-      <c r="E148" s="10"/>
+      <c r="E148" s="9"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
-      <c r="E149" s="10"/>
+      <c r="E149" s="9"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="3"/>
       <c r="D150" s="3"/>
-      <c r="E150" s="10"/>
+      <c r="E150" s="9"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
-      <c r="E151" s="10"/>
+      <c r="E151" s="9"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
-      <c r="E152" s="10"/>
+      <c r="E152" s="9"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="3"/>
       <c r="D153" s="3"/>
-      <c r="E153" s="10"/>
+      <c r="E153" s="9"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
-      <c r="E154" s="10"/>
+      <c r="E154" s="9"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
-      <c r="E155" s="10"/>
+      <c r="E155" s="9"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
-      <c r="E156" s="10"/>
+      <c r="E156" s="9"/>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="3"/>
       <c r="D157" s="3"/>
-      <c r="E157" s="10"/>
+      <c r="E157" s="9"/>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="3"/>
       <c r="D158" s="3"/>
-      <c r="E158" s="10"/>
+      <c r="E158" s="9"/>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
-      <c r="E159" s="10"/>
+      <c r="E159" s="9"/>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
-      <c r="E160" s="10"/>
+      <c r="E160" s="9"/>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="3"/>
       <c r="D161" s="3"/>
-      <c r="E161" s="10"/>
+      <c r="E161" s="9"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="3"/>
       <c r="D162" s="3"/>
-      <c r="E162" s="10"/>
+      <c r="E162" s="9"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
-      <c r="E163" s="10"/>
+      <c r="E163" s="9"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
-      <c r="E164" s="10"/>
+      <c r="E164" s="9"/>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="3"/>
       <c r="D165" s="3"/>
-      <c r="E165" s="10"/>
+      <c r="E165" s="9"/>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="3"/>
       <c r="D166" s="3"/>
-      <c r="E166" s="10"/>
+      <c r="E166" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="B2:E2">
-    <cfRule type="expression" dxfId="10" priority="24">
+    <cfRule type="expression" dxfId="13" priority="24">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2">
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="12" priority="10">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="11" priority="4">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="9" priority="2">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>